<commit_message>
ADD: Created more use cases and added more label printing functionality
</commit_message>
<xml_diff>
--- a/test_doc.xlsx
+++ b/test_doc.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jones\projects\PrintFlo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B17A9DE2-D55C-4961-96C5-03692EB0FFA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{000024FC-895E-48CA-A4D5-C48CCF64EDF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="29020" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,9 +46,6 @@
     <t>Batch</t>
   </si>
   <si>
-    <t>No of Pal/Bag(s)</t>
-  </si>
-  <si>
     <t>Total Qty</t>
   </si>
   <si>
@@ -107,6 +104,9 @@
   </si>
   <si>
     <t>CTEURY38783</t>
+  </si>
+  <si>
+    <t>No Of Pal/Bag(s)</t>
   </si>
 </sst>
 </file>
@@ -655,53 +655,53 @@
   </cellStyles>
   <dxfs count="14">
     <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="25" formatCode="hh:mm"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
           <bgColor theme="9" tint="-0.249977111117893"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="25" formatCode="hh:mm"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -717,21 +717,21 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{BF003C43-C7E3-4794-814C-68B4BE31B51C}" name="Table2" displayName="Table2" ref="A2:L4" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{BF003C43-C7E3-4794-814C-68B4BE31B51C}" name="Table2" displayName="Table2" ref="A2:L4" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
   <autoFilter ref="A2:L4" xr:uid="{BF003C43-C7E3-4794-814C-68B4BE31B51C}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{9CC395E0-F8B2-4A9C-B391-B4D22CA30C46}" name="Date" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{3E3BC55B-0C28-42AB-AC16-0A04604F56B9}" name="Time In" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{F4723BF7-B8E9-4011-85B6-B26A1BDBA040}" name="Container/Truck No" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{88F5F73F-CF33-4862-B031-653733EDCDCB}" name="Product" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{296B1850-D30B-4C63-A3B0-8BA85328E7F4}" name="Supplier" dataDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{2B6C0AC2-9547-4E44-85A6-73523922448E}" name="PO" dataDxfId="8"/>
-    <tableColumn id="7" xr3:uid="{DBE020D5-9A11-4B7F-8563-FD20BEDDEB26}" name="Origin" dataDxfId="7"/>
-    <tableColumn id="8" xr3:uid="{1278ADAC-62A3-4E12-AB9B-0A5D0BD32AC9}" name="Batch" dataDxfId="6"/>
-    <tableColumn id="9" xr3:uid="{FC35A4E9-F4EB-4DA0-BF1F-41B2318693B6}" name="No of Pal/Bag(s)" dataDxfId="5"/>
-    <tableColumn id="10" xr3:uid="{BCE16604-19D1-410C-B9B5-E71001F522BC}" name="Total Qty" dataDxfId="4"/>
-    <tableColumn id="11" xr3:uid="{52C13071-34BE-4B3F-A142-37EDC7C0C3B5}" name="Status" dataDxfId="3"/>
-    <tableColumn id="12" xr3:uid="{9C8968F5-403E-42C1-A92C-3215F0C1FBEB}" name="Storage Loc" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{9CC395E0-F8B2-4A9C-B391-B4D22CA30C46}" name="Date" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{3E3BC55B-0C28-42AB-AC16-0A04604F56B9}" name="Time In" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{F4723BF7-B8E9-4011-85B6-B26A1BDBA040}" name="Container/Truck No" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{88F5F73F-CF33-4862-B031-653733EDCDCB}" name="Product" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{296B1850-D30B-4C63-A3B0-8BA85328E7F4}" name="Supplier" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{2B6C0AC2-9547-4E44-85A6-73523922448E}" name="PO" dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{DBE020D5-9A11-4B7F-8563-FD20BEDDEB26}" name="Origin" dataDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{1278ADAC-62A3-4E12-AB9B-0A5D0BD32AC9}" name="Batch" dataDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{FC35A4E9-F4EB-4DA0-BF1F-41B2318693B6}" name="No Of Pal/Bag(s)" dataDxfId="3"/>
+    <tableColumn id="10" xr3:uid="{BCE16604-19D1-410C-B9B5-E71001F522BC}" name="Total Qty" dataDxfId="2"/>
+    <tableColumn id="11" xr3:uid="{52C13071-34BE-4B3F-A142-37EDC7C0C3B5}" name="Status" dataDxfId="1"/>
+    <tableColumn id="12" xr3:uid="{9C8968F5-403E-42C1-A92C-3215F0C1FBEB}" name="Storage Loc" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1054,7 +1054,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="" visibility="1" width="630" row="4">
+  <wetp:taskpane dockstate="" visibility="1" width="562" row="1">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -1114,16 +1114,16 @@
         <v>7</v>
       </c>
       <c r="I2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="J2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
@@ -1134,34 +1134,34 @@
         <v>0.25</v>
       </c>
       <c r="C3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>13</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>14</v>
       </c>
       <c r="F3" s="3">
         <v>940000568</v>
       </c>
       <c r="G3" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H3" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="I3" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="J3" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K3" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="J3" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="K3" s="3" t="s">
+      <c r="L3" s="3" t="s">
         <v>18</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
@@ -1172,34 +1172,34 @@
         <v>0.25</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D4" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>20</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>21</v>
       </c>
       <c r="F4" s="3">
         <v>940000568</v>
       </c>
       <c r="G4" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="H4" s="3" t="s">
         <v>22</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>23</v>
       </c>
       <c r="I4" s="3">
         <v>20</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K4" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="L4" s="3" t="s">
         <v>18</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
@@ -1210,34 +1210,34 @@
         <v>0.25</v>
       </c>
       <c r="C5" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>26</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>27</v>
       </c>
       <c r="F5" s="3">
         <v>940000568</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I5" s="3">
         <v>20</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="L5" s="3" t="s">
         <v>18</v>
-      </c>
-      <c r="L5" s="3" t="s">
-        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>